<commit_message>
css verbetering  woorden game
</commit_message>
<xml_diff>
--- a/testPlan mbo4 .xlsx
+++ b/testPlan mbo4 .xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:9_{D22523FE-D533-46B6-A69F-E05F62522F18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5749064D-FE0E-403C-847E-13493C7E44C5}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{78096C8C-FED7-427F-812B-0DB23C6C7C8A}"/>
+    <workbookView xWindow="-555" yWindow="2910" windowWidth="21600" windowHeight="11295" xr2:uid="{78096C8C-FED7-427F-812B-0DB23C6C7C8A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -575,7 +575,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -589,41 +589,34 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -651,20 +644,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -684,6 +676,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1014,17 +1010,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18.75">
-      <c r="A1" s="42" t="s">
+      <c r="A1" s="39" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D1" s="44"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="4" t="s">
@@ -1033,15 +1029,15 @@
       <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="39" t="s">
+      <c r="C2" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="39" t="s">
+      <c r="D2" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="G2" s="15"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="6">
@@ -1056,15 +1052,15 @@
       <c r="D3" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="5">
         <v>1.2</v>
       </c>
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="35" t="s">
         <v>6</v>
       </c>
       <c r="C4" s="2" t="s">
@@ -1073,23 +1069,23 @@
       <c r="D4" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="40" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="45"/>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
+      <c r="D5" s="7"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="7">
+      <c r="A6" s="5">
         <v>2.1</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -1101,12 +1097,12 @@
       <c r="D6" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="7">
+      <c r="A7" s="5">
         <v>2.2000000000000002</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -1118,12 +1114,12 @@
       <c r="D7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="15"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
     </row>
     <row r="8" spans="1:7">
-      <c r="A8" s="7">
+      <c r="A8" s="5">
         <v>2.2999999999999998</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -1135,12 +1131,12 @@
       <c r="D8" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="7">
+      <c r="A9" s="5">
         <v>2.4</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -1152,23 +1148,23 @@
       <c r="D9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="15"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="7">
+      <c r="A11" s="5">
         <v>3.1</v>
       </c>
       <c r="B11" s="3" t="s">
@@ -1180,12 +1176,12 @@
       <c r="D11" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="7">
+      <c r="A12" s="5">
         <v>3.2</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -1194,15 +1190,15 @@
       <c r="C12" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="40" t="s">
+      <c r="D12" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="7">
+      <c r="A13" s="5">
         <v>3.3</v>
       </c>
       <c r="B13" s="3" t="s">
@@ -1214,23 +1210,23 @@
       <c r="D13" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="41"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="41"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
+      <c r="B14" s="38"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="7">
+      <c r="A15" s="5">
         <v>4.0999999999999996</v>
       </c>
       <c r="B15" s="2" t="s">
@@ -1242,12 +1238,12 @@
       <c r="D15" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="7">
+      <c r="A16" s="5">
         <v>4.2</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -1259,12 +1255,12 @@
       <c r="D16" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="7">
+      <c r="A17" s="5">
         <v>4.3</v>
       </c>
       <c r="B17" s="2" t="s">
@@ -1276,633 +1272,633 @@
       <c r="D17" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="10"/>
+      <c r="A18" s="8"/>
     </row>
     <row r="19" spans="1:7" ht="24">
-      <c r="A19" s="46"/>
-      <c r="B19" s="46"/>
-      <c r="C19" s="47"/>
-      <c r="D19" s="48" t="s">
+      <c r="A19" s="42"/>
+      <c r="B19" s="42"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="44" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
+      <c r="A20" s="9"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="13"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="14"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
+      <c r="A23" s="12"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="17"/>
-      <c r="B24" s="18"/>
-      <c r="C24" s="22" t="s">
+      <c r="A24" s="15"/>
+      <c r="B24" s="16"/>
+      <c r="C24" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="D24" s="23" t="s">
+      <c r="D24" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="E24" s="24" t="s">
+      <c r="E24" s="21" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="19">
+      <c r="A25" s="17">
         <v>1.1000000000000001</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C25" s="29"/>
-      <c r="D25" s="25" t="s">
+      <c r="C25" s="26"/>
+      <c r="D25" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="E25" s="36"/>
+      <c r="E25" s="33"/>
     </row>
     <row r="26" spans="1:7">
-      <c r="A26" s="19">
+      <c r="A26" s="17">
         <v>1.2</v>
       </c>
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C26" s="30"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="27"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="23"/>
+      <c r="E26" s="24"/>
     </row>
     <row r="27" spans="1:7">
-      <c r="A27" s="19">
+      <c r="A27" s="17">
         <v>2.1</v>
       </c>
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="C27" s="29"/>
-      <c r="D27" s="27" t="s">
+      <c r="C27" s="26"/>
+      <c r="D27" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="E27" s="35"/>
+      <c r="E27" s="32"/>
     </row>
     <row r="28" spans="1:7">
-      <c r="A28" s="19">
+      <c r="A28" s="17">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B28" s="21" t="s">
+      <c r="B28" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="C28" s="29"/>
-      <c r="D28" s="28" t="s">
+      <c r="C28" s="26"/>
+      <c r="D28" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="E28" s="36"/>
+      <c r="E28" s="33"/>
     </row>
     <row r="29" spans="1:7">
-      <c r="A29" s="19">
+      <c r="A29" s="17">
         <v>2.2999999999999998</v>
       </c>
-      <c r="B29" s="21" t="s">
+      <c r="B29" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="C29" s="31"/>
-      <c r="D29" s="27" t="s">
+      <c r="C29" s="28"/>
+      <c r="D29" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="E29" s="35"/>
+      <c r="E29" s="32"/>
     </row>
     <row r="30" spans="1:7">
-      <c r="A30" s="19">
+      <c r="A30" s="17">
         <v>2.4</v>
       </c>
-      <c r="B30" s="21" t="s">
+      <c r="B30" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="C30" s="29"/>
-      <c r="D30" s="28" t="s">
+      <c r="C30" s="26"/>
+      <c r="D30" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="E30" s="36"/>
+      <c r="E30" s="33"/>
     </row>
     <row r="31" spans="1:7">
-      <c r="A31" s="19">
+      <c r="A31" s="17">
         <v>3.1</v>
       </c>
-      <c r="B31" s="21" t="s">
+      <c r="B31" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C31" s="29"/>
-      <c r="D31" s="27" t="s">
+      <c r="C31" s="26"/>
+      <c r="D31" s="24" t="s">
         <v>69</v>
       </c>
-      <c r="E31" s="36"/>
+      <c r="E31" s="33"/>
     </row>
     <row r="32" spans="1:7">
-      <c r="A32" s="19">
+      <c r="A32" s="17">
         <v>3.2</v>
       </c>
-      <c r="B32" s="21" t="s">
+      <c r="B32" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C32" s="29"/>
-      <c r="D32" s="28" t="s">
+      <c r="C32" s="26"/>
+      <c r="D32" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="E32" s="36"/>
+      <c r="E32" s="33"/>
     </row>
     <row r="33" spans="1:5">
-      <c r="A33" s="19">
+      <c r="A33" s="17">
         <v>3.3</v>
       </c>
-      <c r="B33" s="21" t="s">
+      <c r="B33" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="C33" s="29"/>
-      <c r="D33" s="27" t="s">
+      <c r="C33" s="26"/>
+      <c r="D33" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="E33" s="36"/>
+      <c r="E33" s="33"/>
     </row>
     <row r="34" spans="1:5">
-      <c r="A34" s="20">
+      <c r="A34" s="17">
         <v>4.0999999999999996</v>
       </c>
-      <c r="B34" s="21" t="s">
+      <c r="B34" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="C34" s="29"/>
-      <c r="D34" s="28" t="s">
+      <c r="C34" s="26"/>
+      <c r="D34" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="E34" s="36"/>
+      <c r="E34" s="33"/>
     </row>
     <row r="35" spans="1:5">
-      <c r="A35" s="20">
+      <c r="A35" s="17">
         <v>4.2</v>
       </c>
-      <c r="B35" s="21" t="s">
+      <c r="B35" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="C35" s="29"/>
-      <c r="D35" s="27" t="s">
+      <c r="C35" s="26"/>
+      <c r="D35" s="24" t="s">
         <v>68</v>
       </c>
-      <c r="E35" s="36"/>
+      <c r="E35" s="33"/>
     </row>
     <row r="36" spans="1:5">
-      <c r="A36" s="20">
+      <c r="A36" s="17">
         <v>4.3</v>
       </c>
-      <c r="B36" s="19" t="s">
+      <c r="B36" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C36" s="29"/>
-      <c r="D36" s="28" t="s">
+      <c r="C36" s="26"/>
+      <c r="D36" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="E36" s="36"/>
+      <c r="E36" s="33"/>
     </row>
     <row r="41" spans="1:5">
-      <c r="A41" s="11"/>
-      <c r="B41" s="11"/>
-      <c r="C41" s="11"/>
-      <c r="D41" s="11"/>
-      <c r="E41" s="11"/>
+      <c r="A41" s="9"/>
+      <c r="B41" s="9"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
     </row>
     <row r="42" spans="1:5">
-      <c r="A42" s="13" t="s">
+      <c r="A42" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="B42" s="13" t="s">
+      <c r="B42" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C42" s="12" t="s">
+      <c r="C42" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="D42" s="12"/>
-      <c r="E42" s="12"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
     </row>
     <row r="43" spans="1:5">
-      <c r="A43" s="13" t="s">
+      <c r="A43" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="B43" s="13"/>
-      <c r="C43" s="13"/>
-      <c r="D43" s="13"/>
-      <c r="E43" s="13"/>
+      <c r="B43" s="11"/>
+      <c r="C43" s="11"/>
+      <c r="D43" s="11"/>
+      <c r="E43" s="11"/>
     </row>
     <row r="44" spans="1:5">
-      <c r="A44" s="14"/>
-      <c r="B44" s="14"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="14"/>
-      <c r="E44" s="14"/>
+      <c r="A44" s="12"/>
+      <c r="B44" s="12"/>
+      <c r="C44" s="12"/>
+      <c r="D44" s="12"/>
+      <c r="E44" s="12"/>
     </row>
     <row r="45" spans="1:5">
-      <c r="A45" s="17"/>
-      <c r="B45" s="18"/>
-      <c r="C45" s="22" t="s">
+      <c r="A45" s="15"/>
+      <c r="B45" s="16"/>
+      <c r="C45" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="D45" s="23" t="s">
+      <c r="D45" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="E45" s="24" t="s">
+      <c r="E45" s="21" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="46" spans="1:5">
-      <c r="A46" s="19">
+      <c r="A46" s="17">
         <v>1.1000000000000001</v>
       </c>
-      <c r="B46" s="21" t="s">
+      <c r="B46" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C46" s="29"/>
-      <c r="D46" s="32" t="s">
+      <c r="C46" s="26"/>
+      <c r="D46" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="E46" s="35"/>
+      <c r="E46" s="32"/>
     </row>
     <row r="47" spans="1:5">
-      <c r="A47" s="19">
+      <c r="A47" s="17">
         <v>1.2</v>
       </c>
-      <c r="B47" s="21" t="s">
+      <c r="B47" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C47" s="30"/>
-      <c r="D47" s="33" t="s">
+      <c r="C47" s="27"/>
+      <c r="D47" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="E47" s="35"/>
+      <c r="E47" s="32"/>
     </row>
     <row r="48" spans="1:5">
-      <c r="A48" s="19">
+      <c r="A48" s="17">
         <v>2.1</v>
       </c>
-      <c r="B48" s="21" t="s">
+      <c r="B48" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="C48" s="29"/>
-      <c r="D48" s="34" t="s">
+      <c r="C48" s="26"/>
+      <c r="D48" s="31" t="s">
         <v>56</v>
       </c>
-      <c r="E48" s="36"/>
+      <c r="E48" s="33"/>
     </row>
     <row r="49" spans="1:5">
-      <c r="A49" s="19">
+      <c r="A49" s="17">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B49" s="21" t="s">
+      <c r="B49" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="C49" s="29"/>
-      <c r="D49" s="28" t="s">
+      <c r="C49" s="26"/>
+      <c r="D49" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="E49" s="36"/>
+      <c r="E49" s="33"/>
     </row>
     <row r="50" spans="1:5">
-      <c r="A50" s="19">
+      <c r="A50" s="17">
         <v>2.2999999999999998</v>
       </c>
-      <c r="B50" s="21" t="s">
+      <c r="B50" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="C50" s="31"/>
-      <c r="D50" s="27" t="s">
+      <c r="C50" s="28"/>
+      <c r="D50" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="E50" s="36"/>
+      <c r="E50" s="33"/>
     </row>
     <row r="51" spans="1:5">
-      <c r="A51" s="19">
+      <c r="A51" s="17">
         <v>2.4</v>
       </c>
-      <c r="B51" s="21" t="s">
+      <c r="B51" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="C51" s="29"/>
-      <c r="D51" s="28" t="s">
+      <c r="C51" s="26"/>
+      <c r="D51" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="E51" s="36"/>
+      <c r="E51" s="33"/>
     </row>
     <row r="52" spans="1:5">
-      <c r="A52" s="19">
+      <c r="A52" s="17">
         <v>3.1</v>
       </c>
-      <c r="B52" s="21" t="s">
+      <c r="B52" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C52" s="29"/>
-      <c r="D52" s="27" t="s">
+      <c r="C52" s="26"/>
+      <c r="D52" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="E52" s="36"/>
+      <c r="E52" s="33"/>
     </row>
     <row r="53" spans="1:5">
-      <c r="A53" s="19">
+      <c r="A53" s="17">
         <v>3.2</v>
       </c>
-      <c r="B53" s="21" t="s">
+      <c r="B53" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C53" s="29"/>
-      <c r="D53" s="28" t="s">
+      <c r="C53" s="26"/>
+      <c r="D53" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="E53" s="36"/>
+      <c r="E53" s="33"/>
     </row>
     <row r="54" spans="1:5">
-      <c r="A54" s="19">
+      <c r="A54" s="17">
         <v>3.3</v>
       </c>
-      <c r="B54" s="21" t="s">
+      <c r="B54" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="C54" s="29"/>
-      <c r="D54" s="27" t="s">
+      <c r="C54" s="26"/>
+      <c r="D54" s="24" t="s">
         <v>58</v>
       </c>
-      <c r="E54" s="35"/>
+      <c r="E54" s="32"/>
     </row>
     <row r="55" spans="1:5">
-      <c r="A55" s="20">
+      <c r="A55" s="17">
         <v>4.0999999999999996</v>
       </c>
-      <c r="B55" s="21" t="s">
+      <c r="B55" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="C55" s="29"/>
-      <c r="D55" s="28" t="s">
+      <c r="C55" s="26"/>
+      <c r="D55" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="E55" s="36"/>
+      <c r="E55" s="33"/>
     </row>
     <row r="56" spans="1:5">
-      <c r="A56" s="20">
+      <c r="A56" s="17">
         <v>4.2</v>
       </c>
-      <c r="B56" s="21" t="s">
+      <c r="B56" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="C56" s="29"/>
-      <c r="D56" s="27" t="s">
+      <c r="C56" s="26"/>
+      <c r="D56" s="24" t="s">
         <v>59</v>
       </c>
-      <c r="E56" s="36"/>
+      <c r="E56" s="33"/>
     </row>
     <row r="57" spans="1:5">
-      <c r="A57" s="20">
+      <c r="A57" s="17">
         <v>4.3</v>
       </c>
-      <c r="B57" s="19" t="s">
+      <c r="B57" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C57" s="29"/>
-      <c r="D57" s="28" t="s">
+      <c r="C57" s="26"/>
+      <c r="D57" s="25" t="s">
         <v>59</v>
       </c>
-      <c r="E57" s="36"/>
+      <c r="E57" s="33"/>
     </row>
     <row r="61" spans="1:5">
-      <c r="A61" s="11"/>
-      <c r="B61" s="11"/>
-      <c r="C61" s="11"/>
-      <c r="D61" s="11"/>
-      <c r="E61" s="11"/>
+      <c r="A61" s="9"/>
+      <c r="B61" s="9"/>
+      <c r="C61" s="9"/>
+      <c r="D61" s="9"/>
+      <c r="E61" s="9"/>
     </row>
     <row r="62" spans="1:5">
-      <c r="A62" s="13" t="s">
+      <c r="A62" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="B62" s="13" t="s">
+      <c r="B62" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="C62" s="12" t="s">
+      <c r="C62" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="D62" s="12"/>
-      <c r="E62" s="12"/>
+      <c r="D62" s="10"/>
+      <c r="E62" s="10"/>
     </row>
     <row r="63" spans="1:5">
-      <c r="A63" s="13" t="s">
+      <c r="A63" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="B63" s="13"/>
-      <c r="C63" s="13"/>
-      <c r="D63" s="13"/>
-      <c r="E63" s="13"/>
+      <c r="B63" s="11"/>
+      <c r="C63" s="11"/>
+      <c r="D63" s="11"/>
+      <c r="E63" s="11"/>
     </row>
     <row r="64" spans="1:5">
-      <c r="A64" s="14"/>
-      <c r="B64" s="14"/>
-      <c r="C64" s="14"/>
-      <c r="D64" s="14"/>
-      <c r="E64" s="14"/>
+      <c r="A64" s="12"/>
+      <c r="B64" s="12"/>
+      <c r="C64" s="12"/>
+      <c r="D64" s="12"/>
+      <c r="E64" s="12"/>
     </row>
     <row r="65" spans="1:5">
-      <c r="A65" s="17"/>
-      <c r="B65" s="18"/>
-      <c r="C65" s="22" t="s">
+      <c r="A65" s="15"/>
+      <c r="B65" s="16"/>
+      <c r="C65" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="D65" s="23" t="s">
+      <c r="D65" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="E65" s="24" t="s">
+      <c r="E65" s="21" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="66" spans="1:5">
-      <c r="A66" s="19">
+      <c r="A66" s="17">
         <v>1.1000000000000001</v>
       </c>
-      <c r="B66" s="21" t="s">
+      <c r="B66" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="C66" s="37"/>
-      <c r="D66" s="32" t="s">
+      <c r="C66" s="34"/>
+      <c r="D66" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="E66" s="36"/>
+      <c r="E66" s="33"/>
     </row>
     <row r="67" spans="1:5">
-      <c r="A67" s="19">
+      <c r="A67" s="17">
         <v>1.2</v>
       </c>
-      <c r="B67" s="21" t="s">
+      <c r="B67" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="C67" s="30"/>
-      <c r="D67" s="33" t="s">
+      <c r="C67" s="27"/>
+      <c r="D67" s="30" t="s">
         <v>62</v>
       </c>
-      <c r="E67" s="36"/>
+      <c r="E67" s="33"/>
     </row>
     <row r="68" spans="1:5">
-      <c r="A68" s="19">
+      <c r="A68" s="17">
         <v>2.1</v>
       </c>
-      <c r="B68" s="21" t="s">
+      <c r="B68" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="C68" s="29"/>
-      <c r="D68" s="27" t="s">
+      <c r="C68" s="26"/>
+      <c r="D68" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="E68" s="36"/>
+      <c r="E68" s="33"/>
     </row>
     <row r="69" spans="1:5">
-      <c r="A69" s="19">
+      <c r="A69" s="17">
         <v>2.2000000000000002</v>
       </c>
-      <c r="B69" s="21" t="s">
+      <c r="B69" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="C69" s="29"/>
-      <c r="D69" s="28" t="s">
+      <c r="C69" s="26"/>
+      <c r="D69" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="E69" s="36"/>
+      <c r="E69" s="33"/>
     </row>
     <row r="70" spans="1:5">
-      <c r="A70" s="19">
+      <c r="A70" s="17">
         <v>2.2999999999999998</v>
       </c>
-      <c r="B70" s="21" t="s">
+      <c r="B70" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="C70" s="31"/>
-      <c r="D70" s="27" t="s">
+      <c r="C70" s="28"/>
+      <c r="D70" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="E70" s="36"/>
+      <c r="E70" s="33"/>
     </row>
     <row r="71" spans="1:5">
-      <c r="A71" s="19">
+      <c r="A71" s="17">
         <v>2.4</v>
       </c>
-      <c r="B71" s="21" t="s">
+      <c r="B71" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="C71" s="29"/>
-      <c r="D71" s="28" t="s">
+      <c r="C71" s="26"/>
+      <c r="D71" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="E71" s="36"/>
+      <c r="E71" s="33"/>
     </row>
     <row r="72" spans="1:5">
-      <c r="A72" s="19">
+      <c r="A72" s="17">
         <v>3.1</v>
       </c>
-      <c r="B72" s="21" t="s">
+      <c r="B72" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C72" s="29"/>
-      <c r="D72" s="27" t="s">
+      <c r="C72" s="26"/>
+      <c r="D72" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="E72" s="36"/>
+      <c r="E72" s="33"/>
     </row>
     <row r="73" spans="1:5">
-      <c r="A73" s="19">
+      <c r="A73" s="17">
         <v>3.2</v>
       </c>
-      <c r="B73" s="21" t="s">
+      <c r="B73" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C73" s="29"/>
-      <c r="D73" s="28" t="s">
+      <c r="C73" s="26"/>
+      <c r="D73" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="E73" s="36"/>
+      <c r="E73" s="33"/>
     </row>
     <row r="74" spans="1:5">
-      <c r="A74" s="19">
+      <c r="A74" s="17">
         <v>3.3</v>
       </c>
-      <c r="B74" s="21" t="s">
+      <c r="B74" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="C74" s="29"/>
-      <c r="D74" s="27" t="s">
+      <c r="C74" s="26"/>
+      <c r="D74" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="E74" s="35"/>
+      <c r="E74" s="32"/>
     </row>
     <row r="75" spans="1:5">
-      <c r="A75" s="20">
+      <c r="A75" s="17">
         <v>4.0999999999999996</v>
       </c>
-      <c r="B75" s="21" t="s">
+      <c r="B75" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="C75" s="29"/>
-      <c r="D75" s="28" t="s">
+      <c r="C75" s="26"/>
+      <c r="D75" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="E75" s="35"/>
+      <c r="E75" s="32"/>
     </row>
     <row r="76" spans="1:5">
-      <c r="A76" s="20">
+      <c r="A76" s="17">
         <v>4.2</v>
       </c>
-      <c r="B76" s="21" t="s">
+      <c r="B76" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="C76" s="29"/>
-      <c r="D76" s="27" t="s">
+      <c r="C76" s="26"/>
+      <c r="D76" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="E76" s="36"/>
+      <c r="E76" s="33"/>
     </row>
     <row r="77" spans="1:5">
-      <c r="A77" s="20">
+      <c r="A77" s="17">
         <v>4.3</v>
       </c>
-      <c r="B77" s="19" t="s">
+      <c r="B77" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C77" s="29"/>
-      <c r="D77" s="28" t="s">
+      <c r="C77" s="26"/>
+      <c r="D77" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="E77" s="36"/>
+      <c r="E77" s="33"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1911,6 +1907,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="b49b343e-dc06-4710-ae38-80472febd177" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B716430003EDB940A500BB9F8C817975" ma:contentTypeVersion="12" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="b7735c0b3e37f664aea5fcea6d01f028">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="b49b343e-dc06-4710-ae38-80472febd177" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2066ccdfc0cebbb54e956fc3065068d7" ns3:_="">
     <xsd:import namespace="b49b343e-dc06-4710-ae38-80472febd177"/>
@@ -2104,24 +2117,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FEE69F3F-273F-4311-AD97-5077D42E34E0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="b49b343e-dc06-4710-ae38-80472febd177"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="b49b343e-dc06-4710-ae38-80472febd177" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB46FF66-0A0B-424F-808A-A30A62A5BB42}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08B9CE74-93F5-4A09-AA1B-12BD185156F3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2137,28 +2157,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB46FF66-0A0B-424F-808A-A30A62A5BB42}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FEE69F3F-273F-4311-AD97-5077D42E34E0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="b49b343e-dc06-4710-ae38-80472febd177"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>